<commit_message>
fix: align relic effects and preserve dead party members
</commit_message>
<xml_diff>
--- a/outputs/relic-catalog/DiceLand遗物体系表.xlsx
+++ b/outputs/relic-catalog/DiceLand遗物体系表.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="体系总览" sheetId="1" r:id="R3959405528ef4f9f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="遗物完整表" sheetId="2" r:id="Rdb65c5e58d124810"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="体系总览" sheetId="1" r:id="R1a5394d8162840c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="遗物完整表" sheetId="2" r:id="R50fb37bba0554c28"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1101,7 +1101,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="4" t="str">
-        <x:v>2026-10-29。全量配置已更新；本次新增 17 件已核对主要机制，历史备注沿用原记录。未做实战测试。</x:v>
+        <x:v>2026-10-29。159 件当前配置；新增 17 件及 59、138 已核对主要机制，含设计反馈修订。其余历史备注沿用；针对性 EditMode 回归，未完整试玩。</x:v>
       </x:c>
       <x:c r="B5" s="4"/>
       <x:c r="C5" s="4"/>
@@ -1248,7 +1248,7 @@
         <x:v>铁壁徽章、冥龟甲、镜像棱镜、护心盾</x:v>
       </x:c>
       <x:c r="E14" s="14" t="str">
-        <x:v>盾灵逐回合供盾，护甲保养剂开局供盾，安全感强化有盾防御骰，盾反利用失盾反伤。反击刺刃的文案次数限制尚未实现。</x:v>
+        <x:v>盾灵逐回合供盾，护甲保养剂开局供盾，安全感强化有盾防御骰，盾反利用失盾反伤。反击刺刃按每角色每回合一次提供下回合临时强壮。</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="55" customHeight="1">
@@ -1435,7 +1435,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1db9a7373338456e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6290568d4b3241f9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1513,7 +1513,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="4" t="str">
-        <x:v>2026-10-29：159 件当前配置；序号 143–159 已核对主要机制。阴阳鱼实际 ID 为 yin_yang_fish；未做实战测试。</x:v>
+        <x:v>2026-10-29：159 件当前配置；143–159、59、138 已核对主要机制并同步设计反馈。阴阳鱼实际 ID 为 yin_yang_fish；验证为针对性 EditMode 回归。</x:v>
       </x:c>
       <x:c r="B5" s="4"/>
       <x:c r="C5" s="4"/>
@@ -1901,7 +1901,7 @@
         <x:v>杯中没有酒，只有一圈贴着杯壁旋转的金色火舌。</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="44" customHeight="1">
+    <x:row r="19" ht="57" customHeight="1">
       <x:c r="A19" s="8" t="n">
         <x:v>59</x:v>
       </x:c>
@@ -1927,7 +1927,7 @@
         <x:v>即将受到致命伤害</x:v>
       </x:c>
       <x:c r="I19" s="9" t="str">
-        <x:v>敌方燃烧总层数须严格大于5；实现限制为每名角色每场战斗一次，文案未写出。消耗层数取来袭伤害与敌方总燃烧层数的较小值。</x:v>
+        <x:v>敌方燃烧总层数须严格大于 5；满足条件时可反复免受致命伤害，无每场或每回合次数上限。每次消耗层数取来袭伤害与敌方总燃烧层数的较小值；保命后至少剩余 1 点生命，燃烧不足条件时不触发。</x:v>
       </x:c>
       <x:c r="J19" s="9" t="str">
         <x:v>漆黑羽片在火中翻转，灰烬落地前便已长出新的光。</x:v>
@@ -4139,7 +4139,7 @@
         <x:v>获得遗物时</x:v>
       </x:c>
       <x:c r="I92" s="7" t="str">
-        <x:v>效果配置在战斗初始化触发；原文“下一场”与一次性限制需注意，当前未见消耗标记。</x:v>
+        <x:v>获得时将 10×本次获得数量层护盾登记为下一战的全体友方初始状态；进入下一场战斗时消费并清空待发放列表。没有每场持续刷新效果；此前“战斗初始化触发、未见消耗标记”的历史备注已失效。</x:v>
       </x:c>
       <x:c r="J92" s="7" t="str">
         <x:v>贴在胸前时，能听见心跳渐渐平缓。</x:v>
@@ -4171,7 +4171,7 @@
         <x:v>防御骰拼点胜利</x:v>
       </x:c>
       <x:c r="I93" s="9" t="str">
-        <x:v>文案写“每个角色每回合限 1 次”，但当前防御胜利处理器没有回合去重，排队状态还会累加同目标、同延迟的层数。按当前代码，每次防御骰拼点胜利均可排队 1 层临时强壮，延迟到下次回合开始；不能将文案限制视为已实现。</x:v>
+        <x:v>每名角色每回合仅首次防御骰拼点胜利排队获得 1×持有数量层临时强壮，延迟到下次回合开始。去重按本遗物、来源角色与回合计算，该角色更换技能也不能重复领取；不同角色独立计次，新回合及新战斗可再次触发。冥龟甲使用原有不限次效果类型，不受此限制。</x:v>
       </x:c>
       <x:c r="J93" s="9" t="str">
         <x:v>等对手自己撞上来也是一种守株待兔。</x:v>
@@ -4483,7 +4483,7 @@
       </x:c>
       <x:c r="J103" s="9" t="str"/>
     </x:row>
-    <x:row r="104" ht="57" customHeight="1">
+    <x:row r="104" ht="72" customHeight="1">
       <x:c r="A104" s="10" t="n">
         <x:v>153</x:v>
       </x:c>
@@ -4509,7 +4509,7 @@
         <x:v>获得遗物时、战斗建立时</x:v>
       </x:c>
       <x:c r="I104" s="11" t="str">
-        <x:v>获得时实际保留队伍列表第一名，移除其余角色并禁用本局招募；实现并非按初始角色 ID 查找。保留角色的灾厄计算前最大生命 +20×本次获得数量，最终上限仍受灾厄规则影响。每场开局向存活友方施加各 3×持有数量层强壮与重防。</x:v>
+        <x:v>初始角色固定处于队伍首位，阵亡后仍应保留原位。获得时保留首位角色、移除其余角色并禁用本局招募；战斗结算按成员身份更新原队列，保留未参战的阵亡成员。保留角色的灾厄计算前最大生命 +20×本次获得数量，最终上限仍受灾厄规则影响。每场开局向存活友方施加各 3×持有数量层强壮与重防。</x:v>
       </x:c>
       <x:c r="J104" s="11" t="str">
         <x:v>再也不见。</x:v>
@@ -4751,7 +4751,7 @@
         <x:v>玩家拼点失败</x:v>
       </x:c>
       <x:c r="I112" s="11" t="str">
-        <x:v>仅技能原始 energyCost&gt;0 时生效，返还共享能量 1 点。去重键包含本遗物、当前回合、来源角色与技能资产，因此不同角色使用同一技能分别计次；同一技能的多颗骰子不会重复返还。正常战斗遭遇内每场重新计次。</x:v>
+        <x:v>仅技能原始 energyCost&gt;0 时生效，返还共享能量 1 点。设计约定：不同角色拥有的技能视为不同技能，因此按遗物、角色、技能资产、回合分别计次；同一角色同一技能的多颗骰子不会重复返还。正常战斗遭遇内每场重新计次。</x:v>
       </x:c>
       <x:c r="J112" s="11" t="str">
         <x:v>有时付出与回报并不相称，至少这能让你回一些本。</x:v>
@@ -6248,7 +6248,7 @@
         <x:v>概率幸运</x:v>
       </x:c>
       <x:c r="F162" s="13" t="str">
-        <x:v>回合开始时，友方角色有 25% 的几率获得 1 层幸运。</x:v>
+        <x:v>回合开始时，每名存活友方角色独立有 25% 的几率获得 1 层幸运。</x:v>
       </x:c>
       <x:c r="G162" s="13" t="str">
         <x:v>幸运、概率、回合开始</x:v>
@@ -6257,7 +6257,7 @@
         <x:v>战斗回合开始</x:v>
       </x:c>
       <x:c r="I162" s="13" t="str">
-        <x:v>每回合对该效果统一进行一次 25% 概率判定；成功后向所有存活友方各施加 1×持有数量层幸运。不是每名角色独立掷 25%，也没有保底。</x:v>
+        <x:v>回合开始时，每名存活友方角色分别独立进行一次 25% 概率判定；该角色成功时获得 1×持有数量层幸运。未存活角色不判定，不再使用整队共用一次的概率门控，也没有保底。</x:v>
       </x:c>
       <x:c r="J162" s="13" t="str">
         <x:v>许多人梦寐以求的灵药，省着点用。</x:v>
@@ -6280,7 +6280,7 @@
         <x:v>首次伤害强化</x:v>
       </x:c>
       <x:c r="F163" s="13" t="str">
-        <x:v>每场战斗对敌方目标造成的首次伤害翻倍。</x:v>
+        <x:v>每场战斗对敌方目标造成的首次伤害 +100%。</x:v>
       </x:c>
       <x:c r="G163" s="13" t="str">
         <x:v>伤害、首次、每场战斗</x:v>
@@ -6289,7 +6289,7 @@
         <x:v>即将造成伤害</x:v>
       </x:c>
       <x:c r="I163" s="13" t="str">
-        <x:v>每场战斗整支队伍对敌人的第一次正数伤害触发，不是对每个敌人各一次。加入 +100% 伤害百分比修正，与其他百分比来源走统一结算；当前实现不按持有数量放大。非敌方目标或非正数伤害不消耗该次机会。</x:v>
+        <x:v>每场战斗整支队伍首次向敌人结算正数待伤害时，加入 +100% 伤害百分比修正，与其他百分比增伤相加，不是对最终伤害再乘 2；并非对每个敌人各一次。该机会在伤害结算前登记，后续减免不影响已经消耗的首次机会；当前实现不按持有数量放大。</x:v>
       </x:c>
       <x:c r="J163" s="13" t="str">
         <x:v>冷不丁邦邦两棒！</x:v>
@@ -6393,7 +6393,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R29e91901d7314a50"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab2e1a9b0bf44a13"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
balance: reduce damage mitigation on five relics
</commit_message>
<xml_diff>
--- a/outputs/relic-catalog/DiceLand遗物体系表.xlsx
+++ b/outputs/relic-catalog/DiceLand遗物体系表.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="体系总览" sheetId="1" r:id="R1a5394d8162840c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="遗物完整表" sheetId="2" r:id="R50fb37bba0554c28"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="体系总览" sheetId="1" r:id="R2feb1c4a5f5f4fc4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="遗物完整表" sheetId="2" r:id="R3e503db2216d4981"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1101,7 +1101,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="4" t="str">
-        <x:v>2026-10-29。159 件当前配置；新增 17 件及 59、138 已核对主要机制，含设计反馈修订。其余历史备注沿用；针对性 EditMode 回归，未完整试玩。</x:v>
+        <x:v>2026-10-29。159 件当前配置；新增 17 件及 7 件历史遗物已核对主要机制，含本次五件减伤调整。其余历史备注沿用；编辑器验证，未完整试玩。</x:v>
       </x:c>
       <x:c r="B5" s="4"/>
       <x:c r="C5" s="4"/>
@@ -1435,7 +1435,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6290568d4b3241f9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb1b73df1df34ccf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1513,7 +1513,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="4" t="str">
-        <x:v>2026-10-29：159 件当前配置；143–159、59、138 已核对主要机制并同步设计反馈。阴阳鱼实际 ID 为 yin_yang_fish；验证为针对性 EditMode 回归。</x:v>
+        <x:v>2026-10-29：159 件当前配置；143–159 及 12、19、30、59、112、134、138 已核对主要机制并同步调整。阴阳鱼实际 ID 为 yin_yang_fish；验证为针对性 EditMode 回归。</x:v>
       </x:c>
       <x:c r="B5" s="4"/>
       <x:c r="C5" s="4"/>
@@ -2135,7 +2135,7 @@
         <x:v>寒冷减伤</x:v>
       </x:c>
       <x:c r="F26" s="11" t="str">
-        <x:v>友方角色受到攻击时，若敌人拥有寒冷状态，伤害 -20%</x:v>
+        <x:v>友方角色受到攻击时，若敌人拥有寒冷状态，伤害 -10%</x:v>
       </x:c>
       <x:c r="G26" s="11" t="str">
         <x:v>寒冷、寒冷减伤</x:v>
@@ -2143,7 +2143,9 @@
       <x:c r="H26" s="11" t="str">
         <x:v>即将受到攻击伤害</x:v>
       </x:c>
-      <x:c r="I26" s="11" t="str"/>
+      <x:c r="I26" s="11" t="str">
+        <x:v>攻击伤害结算前，攻击者具有至少 1 层寒冷时，伤害减免为 10%×持有数量；只读取攻击者自身的寒冷状态。与同阶段其他百分比减伤相加。</x:v>
+      </x:c>
       <x:c r="J26" s="11" t="str">
         <x:v>护符贴近胸口时仍像雪一样冷，替佩戴者听见冰层下的脚步。</x:v>
       </x:c>
@@ -2707,7 +2709,7 @@
         <x:v>中毒减伤</x:v>
       </x:c>
       <x:c r="F45" s="9" t="str">
-        <x:v>中毒的目标造成伤害 -15%</x:v>
+        <x:v>中毒的目标造成伤害 -10%</x:v>
       </x:c>
       <x:c r="G45" s="9" t="str">
         <x:v>中毒、中毒减伤</x:v>
@@ -2715,7 +2717,9 @@
       <x:c r="H45" s="9" t="str">
         <x:v>即将受到攻击伤害</x:v>
       </x:c>
-      <x:c r="I45" s="9" t="str"/>
+      <x:c r="I45" s="9" t="str">
+        <x:v>攻击伤害结算前，攻击者具有至少 1 层中毒时，伤害减免为 10%×持有数量；只读取攻击者自身的中毒状态。与同阶段其他百分比减伤相加。</x:v>
+      </x:c>
       <x:c r="J45" s="9" t="str">
         <x:v>病了，就会没力气，而这份档案的内容足以致人虚脱。</x:v>
       </x:c>
@@ -3402,15 +3406,17 @@
         <x:v>电流减伤</x:v>
       </x:c>
       <x:c r="F68" s="11" t="str">
-        <x:v>友方角色受到具有电流状态的目标攻击时，受到伤害 -20%</x:v>
+        <x:v>友方角色受到具有电流状态的目标攻击时，受到伤害 -10%</x:v>
       </x:c>
       <x:c r="G68" s="11" t="str">
         <x:v>电流、电流减伤</x:v>
       </x:c>
       <x:c r="H68" s="11" t="str">
-        <x:v>即将受到伤害</x:v>
-      </x:c>
-      <x:c r="I68" s="11" t="str"/>
+        <x:v>即将受到攻击伤害</x:v>
+      </x:c>
+      <x:c r="I68" s="11" t="str">
+        <x:v>攻击伤害结算前，攻击者具有至少 1 层电流时，伤害减免为 10%×持有数量，与同阶段其他百分比减伤相加。已将原本与处理器不匹配的通用受伤触发改为攻击伤害触发，使配置效果实际生效。</x:v>
+      </x:c>
       <x:c r="J68" s="11" t="str">
         <x:v>在里面时感觉格外的安全。</x:v>
       </x:c>
@@ -3737,7 +3743,7 @@
         <x:v>高速减伤</x:v>
       </x:c>
       <x:c r="F79" s="9" t="str">
-        <x:v>若即将对友方角色造成伤害的敌人速度低于友方角色，则使即将到来的伤害 -30%</x:v>
+        <x:v>若即将对友方角色造成伤害的敌人速度低于友方角色，则使即将到来的伤害 -20%</x:v>
       </x:c>
       <x:c r="G79" s="9" t="str">
         <x:v>速度与行动、高速减伤</x:v>
@@ -3745,7 +3751,9 @@
       <x:c r="H79" s="9" t="str">
         <x:v>即将受到攻击伤害</x:v>
       </x:c>
-      <x:c r="I79" s="9" t="str"/>
+      <x:c r="I79" s="9" t="str">
+        <x:v>攻击伤害结算前，来袭敌人的速度严格低于受击友方时，伤害减免为 20%×持有数量；速度相等时不触发。同一结算阶段的百分比减伤相加，合计最多将伤害减至 0。</x:v>
+      </x:c>
       <x:c r="J79" s="9" t="str">
         <x:v>它不追逐时间，只在缝隙里轻轻拨动结局</x:v>
       </x:c>
@@ -3797,7 +3805,7 @@
         <x:v>高速减伤</x:v>
       </x:c>
       <x:c r="F81" s="9" t="str">
-        <x:v>友方角色速度大于 5 时，所受伤害 -30%</x:v>
+        <x:v>友方角色速度大于 5 时，所受伤害 -20%</x:v>
       </x:c>
       <x:c r="G81" s="9" t="str">
         <x:v>速度与行动、高速减伤</x:v>
@@ -3805,7 +3813,9 @@
       <x:c r="H81" s="9" t="str">
         <x:v>即将受到伤害</x:v>
       </x:c>
-      <x:c r="I81" s="9" t="str"/>
+      <x:c r="I81" s="9" t="str">
+        <x:v>进入通用受伤结算时，受击角色速度严格大于 5 才生效，减伤为 20%×持有数量；速度等于 5 时不触发。同一结算阶段的百分比减伤相加。</x:v>
+      </x:c>
       <x:c r="J81" s="9" t="str">
         <x:v>当步伐快到足以融入阴影，再精准的刀锋也会失去准头。</x:v>
       </x:c>
@@ -6393,7 +6403,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab2e1a9b0bf44a13"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3e85627bf4304ccc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>